<commit_message>
feat(master): support Master Project (4 Cr) vs Thesis (16 Cr), PDF evaluation sheets, sorting filters, and comprehensive presentation seed dataset
</commit_message>
<xml_diff>
--- a/backend/excel-templates/New-Test-data/master_all_programs_theses_test_data.xlsx
+++ b/backend/excel-templates/New-Test-data/master_all_programs_theses_test_data.xlsx
@@ -397,272 +397,299 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:J9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="B1" t="str">
         <v>Name</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>Roll</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Title</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Batch</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Cluster</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Program</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Supervisor</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>External_mid_term</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>External_final</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>Thesis</v>
+      </c>
+      <c r="B2" t="str">
         <v>Milan Parajuli</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
         <v>083MSNCS01</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Analysis of Ransomware Attack Vectors and Mitigation Strategies</v>
       </c>
-      <c r="D2" t="str">
-        <v>083</v>
-      </c>
       <c r="E2" t="str">
+        <v>083</v>
+      </c>
+      <c r="F2" t="str">
         <v>Computer networks and security</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>MSNCS</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Prof. Dr. Dinesh Koirala</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>Dr. Prajwal Ghimire</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>Dr. Anisha Rana</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>Project</v>
+      </c>
+      <c r="B3" t="str">
         <v>Nirmaya Bastola</v>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" t="str">
         <v>083MSNCS02</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>AI-Powered Intrusion Detection System for Campus Networks</v>
       </c>
-      <c r="D3" t="str">
-        <v>083</v>
-      </c>
       <c r="E3" t="str">
+        <v>083</v>
+      </c>
+      <c r="F3" t="str">
         <v>Computer networks and security</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>MSNCS</v>
       </c>
-      <c r="G3" t="str">
-        <v>Assoc. Prof. Dr. Meena Shrestha</v>
-      </c>
       <c r="H3" t="str">
-        <v>Dr. Bidur Khadka</v>
+        <v/>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
         <v>Assoc. Prof. Dr. Manisha Aryal</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>Thesis</v>
+      </c>
+      <c r="B4" t="str">
         <v>Oshan Kumal</v>
       </c>
-      <c r="B4" t="str">
+      <c r="C4" t="str">
         <v>083MSICE01</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>5G Massive MIMO Beamforming Optimization Using Machine Learning</v>
       </c>
-      <c r="D4" t="str">
-        <v>083</v>
-      </c>
       <c r="E4" t="str">
+        <v>083</v>
+      </c>
+      <c r="F4" t="str">
         <v>Electronic devices, circuits and communication</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>MSICE</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Dr. Kiran Adhikari</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>Prof. Dr. Lokendra Dhakal</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>Dr. Sabin Wagle</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>Project</v>
+      </c>
+      <c r="B5" t="str">
         <v>Purnima Timalsina</v>
       </c>
-      <c r="B5" t="str">
+      <c r="C5" t="str">
         <v>083MSICE02</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>Performance Evaluation of Cognitive Radio Networks in Dense Urban Areas</v>
       </c>
-      <c r="D5" t="str">
-        <v>083</v>
-      </c>
       <c r="E5" t="str">
+        <v>083</v>
+      </c>
+      <c r="F5" t="str">
         <v>Electronic devices, circuits and communication</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>MSICE</v>
       </c>
-      <c r="G5" t="str">
-        <v>Assoc. Prof. Dr. Gyanendra Thapa</v>
-      </c>
       <c r="H5" t="str">
-        <v>Dr. Prajwal Ghimire</v>
+        <v/>
       </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
         <v>Dr. Anisha Rana</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Thesis</v>
+      </c>
+      <c r="B6" t="str">
         <v>Rajan Dangol</v>
       </c>
-      <c r="B6" t="str">
+      <c r="C6" t="str">
         <v>083MSDSA01</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>Predictive Analytics for Dengue Outbreak Forecasting in Nepal Using LSTM</v>
       </c>
-      <c r="D6" t="str">
-        <v>083</v>
-      </c>
       <c r="E6" t="str">
+        <v>083</v>
+      </c>
+      <c r="F6" t="str">
         <v>AI/ML and image processing</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>MSDSA</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>Dr. Nilima Joshi</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>Assoc. Prof. Dr. Manisha Aryal</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>Dr. Bidur Khadka</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>Project</v>
+      </c>
+      <c r="B7" t="str">
         <v>Sabita Acharya</v>
       </c>
-      <c r="B7" t="str">
+      <c r="C7" t="str">
         <v>083MSDSA02</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>Nepali Sentiment Analysis on Social Media Using Transformer Architectures</v>
       </c>
-      <c r="D7" t="str">
-        <v>083</v>
-      </c>
       <c r="E7" t="str">
-        <v>Audio, NLP and data/text analytics</v>
+        <v>083</v>
       </c>
       <c r="F7" t="str">
+        <v>AI/ML and image processing</v>
+      </c>
+      <c r="G7" t="str">
         <v>MSDSA</v>
       </c>
-      <c r="G7" t="str">
-        <v>Prof. Dr. Raju Poudel</v>
-      </c>
       <c r="H7" t="str">
-        <v>Dr. Sabin Wagle</v>
+        <v/>
       </c>
       <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
         <v>Prof. Dr. Lokendra Dhakal</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>Thesis</v>
+      </c>
+      <c r="B8" t="str">
         <v>Tej Dahal</v>
       </c>
-      <c r="B8" t="str">
+      <c r="C8" t="str">
         <v>083MSCSK01</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>Knowledge Graph Construction for Nepali Biomedical Literature</v>
       </c>
-      <c r="D8" t="str">
-        <v>083</v>
-      </c>
       <c r="E8" t="str">
+        <v>083</v>
+      </c>
+      <c r="F8" t="str">
         <v>Audio, NLP and data/text analytics</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>MSCSK</v>
       </c>
-      <c r="G8" t="str">
+      <c r="H8" t="str">
         <v>Prof. Dr. Dinesh Koirala</v>
       </c>
-      <c r="H8" t="str">
+      <c r="I8" t="str">
         <v>Dr. Prajwal Ghimire</v>
       </c>
-      <c r="I8" t="str">
+      <c r="J8" t="str">
         <v>Dr. Anisha Rana</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>Project</v>
+      </c>
+      <c r="B9" t="str">
         <v>Uma Lama</v>
       </c>
-      <c r="B9" t="str">
+      <c r="C9" t="str">
         <v>083MSCSK02</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
         <v>Automated Semantic Question Answering System Using Ontologies</v>
       </c>
-      <c r="D9" t="str">
-        <v>083</v>
-      </c>
       <c r="E9" t="str">
-        <v>AI/ML and image processing</v>
+        <v>083</v>
       </c>
       <c r="F9" t="str">
+        <v>Audio, NLP and data/text analytics</v>
+      </c>
+      <c r="G9" t="str">
         <v>MSCSK</v>
       </c>
-      <c r="G9" t="str">
-        <v>Assoc. Prof. Dr. Meena Shrestha</v>
-      </c>
       <c r="H9" t="str">
-        <v>Dr. Bidur Khadka</v>
+        <v/>
       </c>
       <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
         <v>Assoc. Prof. Dr. Manisha Aryal</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>